<commit_message>
운동프로그램 갱신 2026-08-11  9:02:37.23
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v10.xlsx
+++ b/운동프로그램_6일_v10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="11_22C8A7C46CBC8E52644F85CDDE579FA68A117E6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C99F1881-B4AB-430F-9D69-F054231E2425}"/>
+  <xr:revisionPtr revIDLastSave="144" documentId="11_22C8A7C46CBC8E52644F85CDDE579FA68A117E6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C836EF99-4C46-4D0F-B521-8204493BC93F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19180,7 +19180,7 @@
       </c>
       <c r="B22" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A22)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A22)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A22)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A22)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A22)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A22)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C22" s="74">
         <f ca="1">SUMIFS(간접계수맵!$F$7:$F$51,간접계수맵!$C$7:$C$51,$A22)</f>
@@ -19188,11 +19188,11 @@
       </c>
       <c r="D22" s="75">
         <f t="shared" ca="1" si="0"/>
-        <v>9.31</v>
+        <v>10.31</v>
       </c>
       <c r="E22" s="7" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>하한</v>
+        <v>충분</v>
       </c>
       <c r="F22" s="73" t="s">
         <v>478</v>
@@ -19255,12 +19255,12 @@
       </c>
       <c r="B25" s="15">
         <f>SUM(B5:B24)</f>
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C25" s="80"/>
       <c r="D25" s="81">
         <f ca="1">SUM(D5:D24)</f>
-        <v>199.69</v>
+        <v>200.69</v>
       </c>
       <c r="E25" s="80" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21468,7 +21468,7 @@
       <c r="B5" s="18"/>
       <c r="C5" s="21">
         <f>월_당기기A!$J$15+화_밀기A!$J$26+수_하체A!$J$22+목_당기기B!$J$14+금_밀기B!$J$29+토_하체B!$J$23</f>
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>57</v>
@@ -21865,7 +21865,7 @@
       </c>
       <c r="E8" s="30">
         <f>목_당기기B!$E$14</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F8" s="27" t="s">
         <v>104</v>
@@ -21942,7 +21942,7 @@
       <c r="D12" s="35"/>
       <c r="E12" s="34">
         <f>SUM(E5:E11)</f>
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
@@ -23570,7 +23570,7 @@
         <v>10</v>
       </c>
       <c r="E11" s="27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="33" t="s">
         <v>199</v>
@@ -23584,7 +23584,7 @@
       </c>
       <c r="J11" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K11,$E11,0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" s="42">
         <v>1</v>
@@ -23666,11 +23666,11 @@
       </c>
       <c r="E14" s="34">
         <f>SUM(E6:E13)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J14" s="41">
         <f>SUM(J6:J13)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-08-11 14:41:09.85
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v10.xlsx
+++ b/운동프로그램_6일_v10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="144" documentId="11_22C8A7C46CBC8E52644F85CDDE579FA68A117E6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C836EF99-4C46-4D0F-B521-8204493BC93F}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="11_22C8A7C46CBC8E52644F85CDDE579FA68A117E6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A7894A9-A8A7-48E9-81C1-6FBEF30ED0C6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -16897,11 +16897,11 @@
         <v>20</v>
       </c>
       <c r="D9" s="4">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="E9" s="9">
         <f>INDEX(증량기록!$G$10:$G$21,$C$4)</f>
-        <v>22.25</v>
+        <v>24.75</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>11</v>
@@ -17085,7 +17085,7 @@
       </c>
       <c r="D40" s="9">
         <f>증량기록!G10</f>
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="E40" s="9">
         <f>증량기록!I10</f>
@@ -17106,7 +17106,7 @@
       </c>
       <c r="D41" s="16">
         <f>증량기록!G11</f>
-        <v>22.25</v>
+        <v>24.75</v>
       </c>
       <c r="E41" s="16">
         <f>증량기록!I11</f>
@@ -17127,7 +17127,7 @@
       </c>
       <c r="D42" s="16">
         <f>증량기록!G12</f>
-        <v>24.5</v>
+        <v>27</v>
       </c>
       <c r="E42" s="16">
         <f>증량기록!I12</f>
@@ -17148,7 +17148,7 @@
       </c>
       <c r="D43" s="16">
         <f>증량기록!G13</f>
-        <v>26.75</v>
+        <v>29.25</v>
       </c>
       <c r="E43" s="16">
         <f>증량기록!I13</f>
@@ -17169,7 +17169,7 @@
       </c>
       <c r="D44" s="16">
         <f>증량기록!G14</f>
-        <v>29</v>
+        <v>31.5</v>
       </c>
       <c r="E44" s="16">
         <f>증량기록!I14</f>
@@ -17190,7 +17190,7 @@
       </c>
       <c r="D45" s="16">
         <f>증량기록!G15</f>
-        <v>31.25</v>
+        <v>33.75</v>
       </c>
       <c r="E45" s="16">
         <f>증량기록!I15</f>
@@ -17211,7 +17211,7 @@
       </c>
       <c r="D46" s="16">
         <f>증량기록!G16</f>
-        <v>33.5</v>
+        <v>36</v>
       </c>
       <c r="E46" s="16">
         <f>증량기록!I16</f>
@@ -17232,7 +17232,7 @@
       </c>
       <c r="D47" s="16">
         <f>증량기록!G17</f>
-        <v>35.75</v>
+        <v>38.25</v>
       </c>
       <c r="E47" s="16">
         <f>증량기록!I17</f>
@@ -17253,7 +17253,7 @@
       </c>
       <c r="D48" s="16">
         <f>증량기록!G18</f>
-        <v>38</v>
+        <v>40.5</v>
       </c>
       <c r="E48" s="16">
         <f>증량기록!I18</f>
@@ -17274,7 +17274,7 @@
       </c>
       <c r="D49" s="16">
         <f>증량기록!G19</f>
-        <v>40.25</v>
+        <v>42.75</v>
       </c>
       <c r="E49" s="16">
         <f>증량기록!I19</f>
@@ -17295,7 +17295,7 @@
       </c>
       <c r="D50" s="16">
         <f>증량기록!G20</f>
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="E50" s="16">
         <f>증량기록!I20</f>
@@ -17316,7 +17316,7 @@
       </c>
       <c r="D51" s="16">
         <f>증량기록!G21</f>
-        <v>44.75</v>
+        <v>47.25</v>
       </c>
       <c r="E51" s="16">
         <f>증량기록!I21</f>
@@ -19515,7 +19515,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="16">
         <f>시작중량_설정!$D$9</f>
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="16">
@@ -19542,7 +19542,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="16">
         <f t="shared" ref="G11:G21" si="2">IF(H10="X",G10,G10+$C$7)</f>
-        <v>22.25</v>
+        <v>24.75</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="16">
@@ -19569,7 +19569,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="16">
         <f t="shared" si="2"/>
-        <v>24.5</v>
+        <v>27</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="16">
@@ -19596,7 +19596,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="16">
         <f t="shared" si="2"/>
-        <v>26.75</v>
+        <v>29.25</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="16">
@@ -19623,7 +19623,7 @@
       <c r="F14" s="4"/>
       <c r="G14" s="16">
         <f t="shared" si="2"/>
-        <v>29</v>
+        <v>31.5</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="16">
@@ -19650,7 +19650,7 @@
       <c r="F15" s="4"/>
       <c r="G15" s="16">
         <f t="shared" si="2"/>
-        <v>31.25</v>
+        <v>33.75</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="16">
@@ -19677,7 +19677,7 @@
       <c r="F16" s="4"/>
       <c r="G16" s="16">
         <f t="shared" si="2"/>
-        <v>33.5</v>
+        <v>36</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="16">
@@ -19704,7 +19704,7 @@
       <c r="F17" s="4"/>
       <c r="G17" s="16">
         <f t="shared" si="2"/>
-        <v>35.75</v>
+        <v>38.25</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="16">
@@ -19731,7 +19731,7 @@
       <c r="F18" s="4"/>
       <c r="G18" s="16">
         <f t="shared" si="2"/>
-        <v>38</v>
+        <v>40.5</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="16">
@@ -19758,7 +19758,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="16">
         <f t="shared" si="2"/>
-        <v>40.25</v>
+        <v>42.75</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="16">
@@ -19785,7 +19785,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="16">
         <f t="shared" si="2"/>
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="16">
@@ -19812,7 +19812,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="16">
         <f t="shared" si="2"/>
-        <v>44.75</v>
+        <v>47.25</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="16">
@@ -20429,7 +20429,7 @@
       </c>
       <c r="D5" s="94">
         <f>시작중량_설정!$E$9</f>
-        <v>22.25</v>
+        <v>24.75</v>
       </c>
       <c r="E5" s="86">
         <v>5</v>
@@ -22573,9 +22573,9 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1">
-      <c r="A9" s="27" t="str">
+      <c r="A9" s="27">
         <f>IF(MAX(20,MROUND(시작중량_설정!$E$9*0.9,2.5))&lt;=MAX(20,MROUND(시작중량_설정!$E$9*0.75,2.5)),"생략",MAX(20,MROUND(시작중량_설정!$E$9*0.9,2.5)))</f>
-        <v>생략</v>
+        <v>22.5</v>
       </c>
       <c r="B9" s="27">
         <v>2</v>
@@ -22587,7 +22587,7 @@
     <row r="10" spans="1:3" ht="15" customHeight="1">
       <c r="A10" s="47">
         <f>시작중량_설정!$E$9</f>
-        <v>22.25</v>
+        <v>24.75</v>
       </c>
       <c r="B10" s="34">
         <v>5</v>
@@ -22673,7 +22673,7 @@
       </c>
       <c r="D20" s="51">
         <f>시작중량_설정!$E$9</f>
-        <v>22.25</v>
+        <v>24.75</v>
       </c>
       <c r="E20" s="50">
         <v>5</v>

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-08-12  7:44:32.58
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v10.xlsx
+++ b/운동프로그램_6일_v10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="11_22C8A7C46CBC8E52644F85CDDE579FA68A117E6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A7894A9-A8A7-48E9-81C1-6FBEF30ED0C6}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="11_22C8A7C46CBC8E52644F85CDDE579FA68A117E6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2328B29-7BCA-4D36-B1D6-11BE8DF18B97}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -16454,14 +16454,14 @@
     </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -17355,28 +17355,28 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="100" t="s">
+      <c r="A2" s="99" t="s">
         <v>392</v>
       </c>
-      <c r="B2" s="100"/>
-      <c r="C2" s="100"/>
-      <c r="D2" s="100"/>
-      <c r="E2" s="100"/>
-      <c r="F2" s="100"/>
-      <c r="G2" s="100"/>
-      <c r="H2" s="100"/>
+      <c r="B2" s="99"/>
+      <c r="C2" s="99"/>
+      <c r="D2" s="99"/>
+      <c r="E2" s="99"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="99"/>
+      <c r="H2" s="99"/>
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A4" s="101" t="s">
+      <c r="A4" s="100" t="s">
         <v>393</v>
       </c>
-      <c r="B4" s="101"/>
-      <c r="C4" s="101"/>
-      <c r="D4" s="101"/>
-      <c r="E4" s="101"/>
-      <c r="F4" s="101"/>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
+      <c r="B4" s="100"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
+      <c r="H4" s="100"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
       <c r="A6" s="56" t="s">
@@ -17839,11 +17839,11 @@
       </c>
       <c r="E22" s="59">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F22" s="60">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="G22" s="61" t="s">
         <v>403</v>
@@ -18670,7 +18670,7 @@
       </c>
       <c r="F52" s="72">
         <f ca="1">SUM(F7:F51)</f>
-        <v>53.689999999999991</v>
+        <v>55.189999999999991</v>
       </c>
     </row>
   </sheetData>
@@ -18749,7 +18749,7 @@
       <c r="F5" s="73" t="s">
         <v>460</v>
       </c>
-      <c r="G5" s="99" t="s">
+      <c r="G5" s="101" t="s">
         <v>461</v>
       </c>
       <c r="H5" s="76">
@@ -18780,7 +18780,7 @@
       <c r="F6" s="73" t="s">
         <v>462</v>
       </c>
-      <c r="G6" s="99"/>
+      <c r="G6" s="101"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
       <c r="A7" s="73" t="s">
@@ -18805,12 +18805,12 @@
       <c r="F7" s="73" t="s">
         <v>463</v>
       </c>
-      <c r="G7" s="99" t="s">
+      <c r="G7" s="101" t="s">
         <v>464</v>
       </c>
       <c r="H7" s="76">
         <f ca="1">SUM(D7:D10)</f>
-        <v>35.72</v>
+        <v>38.72</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
@@ -18836,7 +18836,7 @@
       <c r="F8" s="73" t="s">
         <v>465</v>
       </c>
-      <c r="G8" s="99"/>
+      <c r="G8" s="101"/>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
       <c r="A9" s="73" t="s">
@@ -18861,7 +18861,7 @@
       <c r="F9" s="73" t="s">
         <v>466</v>
       </c>
-      <c r="G9" s="99"/>
+      <c r="G9" s="101"/>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
       <c r="A10" s="73" t="s">
@@ -18869,7 +18869,7 @@
       </c>
       <c r="B10" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A10)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A10)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A10)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A10)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A10)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A10)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C10" s="74">
         <f ca="1">SUMIFS(간접계수맵!$F$7:$F$51,간접계수맵!$C$7:$C$51,$A10)</f>
@@ -18877,7 +18877,7 @@
       </c>
       <c r="D10" s="75">
         <f t="shared" ca="1" si="0"/>
-        <v>10.32</v>
+        <v>13.32</v>
       </c>
       <c r="E10" s="7" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -18886,7 +18886,7 @@
       <c r="F10" s="73" t="s">
         <v>467</v>
       </c>
-      <c r="G10" s="99"/>
+      <c r="G10" s="101"/>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
       <c r="A11" s="73" t="s">
@@ -18973,11 +18973,11 @@
       </c>
       <c r="C14" s="74">
         <f ca="1">SUMIFS(간접계수맵!$F$7:$F$51,간접계수맵!$C$7:$C$51,$A14)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="D14" s="75">
         <f t="shared" ca="1" si="0"/>
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="E14" s="7" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -19066,7 +19066,7 @@
       <c r="F17" s="73" t="s">
         <v>473</v>
       </c>
-      <c r="G17" s="99" t="s">
+      <c r="G17" s="101" t="s">
         <v>254</v>
       </c>
       <c r="H17" s="76">
@@ -19097,7 +19097,7 @@
       <c r="F18" s="73" t="s">
         <v>474</v>
       </c>
-      <c r="G18" s="99"/>
+      <c r="G18" s="101"/>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1">
       <c r="A19" s="73" t="s">
@@ -19155,7 +19155,7 @@
       </c>
       <c r="B21" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A21)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A21)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A21)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A21)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A21)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A21)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21" s="74">
         <f ca="1">SUMIFS(간접계수맵!$F$7:$F$51,간접계수맵!$C$7:$C$51,$A21)</f>
@@ -19163,7 +19163,7 @@
       </c>
       <c r="D21" s="75">
         <f t="shared" ca="1" si="0"/>
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="E21" s="7" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -19255,12 +19255,12 @@
       </c>
       <c r="B25" s="15">
         <f>SUM(B5:B24)</f>
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C25" s="80"/>
       <c r="D25" s="81">
         <f ca="1">SUM(D5:D24)</f>
-        <v>200.69</v>
+        <v>206.19</v>
       </c>
       <c r="E25" s="80" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21468,7 +21468,7 @@
       <c r="B5" s="18"/>
       <c r="C5" s="21">
         <f>월_당기기A!$J$15+화_밀기A!$J$26+수_하체A!$J$22+목_당기기B!$J$14+금_밀기B!$J$29+토_하체B!$J$23</f>
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>57</v>
@@ -21802,7 +21802,7 @@
       </c>
       <c r="E5" s="27">
         <f>월_당기기A!$E$15</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>104</v>
@@ -21823,7 +21823,7 @@
       </c>
       <c r="E6" s="27">
         <f>화_밀기A!$E$26</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F6" s="27" t="s">
         <v>109</v>
@@ -21942,7 +21942,7 @@
       <c r="D12" s="35"/>
       <c r="E12" s="34">
         <f>SUM(E5:E11)</f>
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
@@ -22270,7 +22270,7 @@
         <v>184</v>
       </c>
       <c r="E9" s="27">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="33" t="s">
         <v>185</v>
@@ -22286,7 +22286,7 @@
       </c>
       <c r="J9" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K9,$E9,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K9" s="42">
         <v>1</v>
@@ -22474,11 +22474,11 @@
       </c>
       <c r="E15" s="45">
         <f>SUM(E6:E14)</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J15" s="46">
         <f>SUM(J6:J14)</f>
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -22782,7 +22782,7 @@
         <v>190</v>
       </c>
       <c r="E23" s="27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F23" s="33" t="s">
         <v>173</v>
@@ -22796,7 +22796,7 @@
       </c>
       <c r="J23" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K23,$E23,0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K23" s="42">
         <v>1</v>
@@ -22872,11 +22872,11 @@
       </c>
       <c r="E26" s="34">
         <f>SUM(E20:E25)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J26" s="41">
         <f>SUM(J20:J25)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>